<commit_message>
feat: implement intent classification pipeline with training, evaluation scripts, and a Streamlit UI
</commit_message>
<xml_diff>
--- a/data/processed/SCCU_tfidf_results.xlsx
+++ b/data/processed/SCCU_tfidf_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://claysysin-my.sharepoint.com/personal/anandha_kumar_claysys_in/Documents/Desktop/Code Base/Global search/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_46AD8E42FE17860E93B14421E07AD51646C677E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DA4FCB8-267D-49BD-9E52-C549116F7972}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_46AD8E42FE17860E93B14421E07AD51646C677E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0320301A-C0E5-43F4-AB51-A0AA65AF7125}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="all" sheetId="1" r:id="rId1"/>

</xml_diff>